<commit_message>
samples discription and happy path sample
</commit_message>
<xml_diff>
--- a/samples/sample_1/SAFE_VESSELS_INDEX_20251201.XLSX
+++ b/samples/sample_1/SAFE_VESSELS_INDEX_20251201.XLSX
@@ -1,135 +1,130 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Sheet2" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Sheet3" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
-  <si>
-    <t xml:space="preserve">SHIPID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHIPNAME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CUSTNO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMONO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHIPSTAT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OFFICEEMAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOTE1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOTE2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOTE3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SH_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Big Ship</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CUST_001  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bigdog@email.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brain@email.com</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
+  <si>
+    <t>SHIPID</t>
+  </si>
+  <si>
+    <t>SHIPNAME</t>
+  </si>
+  <si>
+    <t>CUSTNO</t>
+  </si>
+  <si>
+    <t>IMONO</t>
+  </si>
+  <si>
+    <t>SHIPSTAT</t>
+  </si>
+  <si>
+    <t>EMAIL</t>
+  </si>
+  <si>
+    <t>OFFICEEMAIL</t>
+  </si>
+  <si>
+    <t>NOTE1</t>
+  </si>
+  <si>
+    <t>NOTE2</t>
+  </si>
+  <si>
+    <t>NOTE3</t>
+  </si>
+  <si>
+    <t>ship 01</t>
+  </si>
+  <si>
+    <t>eagle</t>
+  </si>
+  <si>
+    <t>cust 001</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>eagle@test.com</t>
+  </si>
+  <si>
+    <t>bird@test.com</t>
   </si>
   <si>
     <t xml:space="preserve">BUN                                                         </t>
   </si>
   <si>
-    <t xml:space="preserve">AMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FUN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SH_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fast Ship</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CUST_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fastdog@email.com</t>
+    <t>AMS</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>ship 02</t>
+  </si>
+  <si>
+    <t>hawk</t>
+  </si>
+  <si>
+    <t>hawk@test.com</t>
+  </si>
+  <si>
+    <t>ship 03</t>
+  </si>
+  <si>
+    <t>falcon</t>
+  </si>
+  <si>
+    <t>9009003</t>
+  </si>
+  <si>
+    <t>falcon@test.com</t>
+  </si>
+  <si>
+    <t>BUN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <charset val="1"/>
+      <color theme="1"/>
+      <family val="2"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
+      <charset val="1"/>
+      <color theme="1"/>
+      <family val="2"/>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -141,7 +136,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -149,57 +144,31 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-  </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -379,25 +348,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="30.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.85"/>
+    <col min="1" max="1" width="15.14" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30.43" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.71" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.3" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.29" style="1" customWidth="1"/>
+    <col min="6" max="6" width="30.71" style="1" customWidth="1"/>
+    <col min="7" max="8" width="30" style="1" customWidth="1"/>
+    <col min="9" max="9" width="30.14" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6.85" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -429,7 +395,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" ht="15" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -439,7 +405,7 @@
       <c r="C2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="1">
         <v>9009001</v>
       </c>
       <c r="E2" s="1" t="s">
@@ -451,17 +417,17 @@
       <c r="G2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>19</v>
       </c>
@@ -469,73 +435,81 @@
         <v>20</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1">
         <v>9009002</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="1" t="s">
         <v>16</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="bigdog@email.com"/>
-    <hyperlink ref="G2" r:id="rId2" display="brain@email"/>
-    <hyperlink ref="F3" r:id="rId3" display="fastdog@email.com"/>
-    <hyperlink ref="G3" r:id="rId4" display="brain@email"/>
+    <hyperlink ref="F2" r:id="rId1"/>
+    <hyperlink ref="G2" r:id="rId2"/>
+    <hyperlink ref="F3" r:id="rId3"/>
+    <hyperlink ref="G3" r:id="rId4"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="1" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <sheetData/>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <sheetData/>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
remove office email from excel ingestion
</commit_message>
<xml_diff>
--- a/samples/sample_1/SAFE_VESSELS_INDEX_20251201.XLSX
+++ b/samples/sample_1/SAFE_VESSELS_INDEX_20251201.XLSX
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
   <si>
     <t xml:space="preserve">SHIPID</t>
   </si>
@@ -42,9 +42,6 @@
     <t xml:space="preserve">EMAIL</t>
   </si>
   <si>
-    <t xml:space="preserve">OFFICEEMAIL</t>
-  </si>
-  <si>
     <t xml:space="preserve">NOTE1</t>
   </si>
   <si>
@@ -66,10 +63,7 @@
     <t xml:space="preserve">A</t>
   </si>
   <si>
-    <t xml:space="preserve">eagle@test.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bird@test.com</t>
+    <t xml:space="preserve">mavi.maths@gmail.com;rsmavi.hb@gmail.com</t>
   </si>
   <si>
     <t xml:space="preserve">BUN                                                         </t>
@@ -84,9 +78,6 @@
     <t xml:space="preserve">hawk</t>
   </si>
   <si>
-    <t xml:space="preserve">hawk@test.com</t>
-  </si>
-  <si>
     <t xml:space="preserve">ship 03</t>
   </si>
   <si>
@@ -97,9 +88,6 @@
   </si>
   <si>
     <t xml:space="preserve">9009003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">falcon@test.com</t>
   </si>
   <si>
     <t xml:space="preserve">BUN</t>
@@ -191,11 +179,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -391,7 +379,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.14"/>
@@ -399,10 +387,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="30.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="47.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="30.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -433,100 +422,87 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>9009001</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>9009002</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="G3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="E4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="eagle@test.com"/>
-    <hyperlink ref="G2" r:id="rId2" display="bird@test.com"/>
-    <hyperlink ref="F3" r:id="rId3" display="hawk@test.com"/>
-    <hyperlink ref="G3" r:id="rId4" display="bird@test.com"/>
+    <hyperlink ref="F2" r:id="rId1" display="mavi.maths@gmail.com"/>
+    <hyperlink ref="F3" r:id="rId2" display="mavi.maths@gmail.com"/>
+    <hyperlink ref="F4" r:id="rId3" display="mavi.maths@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Added optional SMRTCHRT column to vessel index
</commit_message>
<xml_diff>
--- a/samples/sample_1/SAFE_VESSELS_INDEX_20251201.XLSX
+++ b/samples/sample_1/SAFE_VESSELS_INDEX_20251201.XLSX
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
   <si>
     <t xml:space="preserve">SHIPID</t>
   </si>
@@ -51,6 +51,9 @@
     <t xml:space="preserve">NOTE3</t>
   </si>
   <si>
+    <t xml:space="preserve">SMRTCHRT</t>
+  </si>
+  <si>
     <t xml:space="preserve">ship 01</t>
   </si>
   <si>
@@ -70,6 +73,9 @@
   </si>
   <si>
     <t xml:space="preserve">AMS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rajinder@mavi.phd;mavirsep@gmail.com</t>
   </si>
   <si>
     <t xml:space="preserve">ship 02</t>
@@ -174,7 +180,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -183,7 +189,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -379,7 +397,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.14"/>
@@ -391,118 +409,126 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="30.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="40.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="2" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>9009001</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>9009002</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="mavi.maths@gmail.com"/>
-    <hyperlink ref="F3" r:id="rId2" display="mavi.maths@gmail.com"/>
-    <hyperlink ref="F4" r:id="rId3" display="mavi.maths@gmail.com"/>
+    <hyperlink ref="F2" r:id="rId1" display="mavi.maths@gmail.com;rsmavi.hb@gmail.com"/>
+    <hyperlink ref="J2" r:id="rId2" display="rajinder@mavi.phd"/>
+    <hyperlink ref="F3" r:id="rId3" display="mavi.maths@gmail.com;rsmavi.hb@gmail.com"/>
+    <hyperlink ref="F4" r:id="rId4" display="mavi.maths@gmail.com;rsmavi.hb@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>